<commit_message>
Started Testing Oscillators. Starting coding Hill Production reactions. Fixed a bug in the mass action reaction class where the signature was created from the constructor arguments and not the self attributes.
</commit_message>
<xml_diff>
--- a/applications/tracking_disturbance_3species_ppo/Discover_Molecular_Integrators_PPO.xlsx
+++ b/applications/tracking_disturbance_3species_ppo/Discover_Molecular_Integrators_PPO.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="54">
   <si>
     <t>Timestamp</t>
   </si>
@@ -34,6 +34,9 @@
     <t>2025-10-12 21:11:52</t>
   </si>
   <si>
+    <t>2025-10-13 19:25:26</t>
+  </si>
+  <si>
     <t>URL</t>
   </si>
   <si>
@@ -50,6 +53,9 @@
   </si>
   <si>
     <t>https://www.comet.com/maurice-filo/molecular-integrators-ppo/2be6830e3f38494a9684052ea7096d9c</t>
+  </si>
+  <si>
+    <t>https://www.comet.com/maurice-filo/molecular-integrators-ppo/b60487fb4589494fb5ab391ef0ad8fb1</t>
   </si>
   <si>
     <t>Maximum Number of Added Reactions</t>
@@ -571,15 +577,16 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="11" width="36.14785714285715" customWidth="1" bestFit="1"/>
     <col min="2" max="2" style="12" width="21.862142857142857" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="13" width="29.719285714285714" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="13" width="26.433571428571426" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="13" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="14" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -595,36 +602,42 @@
       <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>5</v>
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>6</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="E2" s="3" t="s">
         <v>11</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>13</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B3" s="2">
         <v>5</v>
@@ -638,13 +651,16 @@
       <c r="E3" s="2">
         <v>5</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="2">
+        <v>5</v>
+      </c>
+      <c r="G3" s="6">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B4" s="2">
         <v>3</v>
@@ -658,13 +674,16 @@
       <c r="E4" s="2">
         <v>3</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="2">
+        <v>3</v>
+      </c>
+      <c r="G4" s="6">
         <v>3</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2">
         <v>2</v>
@@ -678,13 +697,16 @@
       <c r="E5" s="2">
         <v>2</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="2">
+        <v>2</v>
+      </c>
+      <c r="G5" s="6">
         <v>2</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B6" s="2">
         <v>1280</v>
@@ -698,13 +720,16 @@
       <c r="E6" s="2">
         <v>1280</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="2">
         <v>1280</v>
+      </c>
+      <c r="G6" s="6">
+        <v>2560</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B7" s="2" t="b">
         <v>0</v>
@@ -715,16 +740,19 @@
       <c r="D7" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="E7" s="8" t="b">
+      <c r="E7" s="7" t="b">
         <v>0</v>
       </c>
-      <c r="F7" s="5" t="b">
+      <c r="F7" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" s="5" t="b">
         <v>0</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B8" s="9">
         <v>0.0001</v>
@@ -738,13 +766,16 @@
       <c r="E8" s="9">
         <v>0.0001</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="9">
+        <v>0.0001</v>
+      </c>
+      <c r="G8" s="10">
         <v>0.0001</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B9" s="2">
         <v>500</v>
@@ -758,13 +789,16 @@
       <c r="E9" s="2">
         <v>500</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="2">
+        <v>500</v>
+      </c>
+      <c r="G9" s="6">
         <v>500</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B10" s="2">
         <v>5</v>
@@ -778,13 +812,16 @@
       <c r="E10" s="2">
         <v>5</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="2">
+        <v>5</v>
+      </c>
+      <c r="G10" s="6">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B11" s="2">
         <v>1024</v>
@@ -798,13 +835,16 @@
       <c r="E11" s="2">
         <v>1024</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="2">
+        <v>1024</v>
+      </c>
+      <c r="G11" s="6">
         <v>1024</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12" s="2">
         <v>10240</v>
@@ -818,13 +858,16 @@
       <c r="E12" s="2">
         <v>10240</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="2">
+        <v>10240</v>
+      </c>
+      <c r="G12" s="6">
         <v>10240</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B13" s="2">
         <v>128</v>
@@ -838,13 +881,16 @@
       <c r="E13" s="2">
         <v>128</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="2">
+        <v>128</v>
+      </c>
+      <c r="G13" s="6">
         <v>128</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B14" s="9">
         <v>0.0001</v>
@@ -858,13 +904,16 @@
       <c r="E14" s="9">
         <v>0.1</v>
       </c>
-      <c r="F14" s="10">
+      <c r="F14" s="9">
         <v>0.1</v>
+      </c>
+      <c r="G14" s="10">
+        <v>0.0001</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15" s="9">
         <v>0.75</v>
@@ -878,13 +927,16 @@
       <c r="E15" s="9">
         <v>0.75</v>
       </c>
-      <c r="F15" s="10">
+      <c r="F15" s="9">
+        <v>0.75</v>
+      </c>
+      <c r="G15" s="10">
         <v>0.75</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16" s="2">
         <v>10000</v>
@@ -898,13 +950,16 @@
       <c r="E16" s="2">
         <v>10000</v>
       </c>
-      <c r="F16" s="6">
+      <c r="F16" s="2">
         <v>50</v>
+      </c>
+      <c r="G16" s="6">
+        <v>5000</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17" s="9">
         <v>0.0001</v>
@@ -918,13 +973,16 @@
       <c r="E17" s="9">
         <v>0.0001</v>
       </c>
-      <c r="F17" s="10">
+      <c r="F17" s="9">
+        <v>0.0001</v>
+      </c>
+      <c r="G17" s="10">
         <v>0.0001</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18" s="9">
         <v>0.99</v>
@@ -938,13 +996,16 @@
       <c r="E18" s="9">
         <v>0.9</v>
       </c>
-      <c r="F18" s="10">
+      <c r="F18" s="9">
         <v>0.9</v>
+      </c>
+      <c r="G18" s="10">
+        <v>0.99</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19" s="2">
         <v>0</v>
@@ -958,13 +1019,16 @@
       <c r="E19" s="2">
         <v>0</v>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
+      <c r="G19" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B20" s="2">
         <v>1</v>
@@ -978,13 +1042,16 @@
       <c r="E20" s="2">
         <v>1</v>
       </c>
-      <c r="F20" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
+      <c r="F20" s="2">
+        <v>1</v>
+      </c>
+      <c r="G20" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B21" s="2">
         <v>20</v>
@@ -998,13 +1065,16 @@
       <c r="E21" s="2">
         <v>20</v>
       </c>
-      <c r="F21" s="6">
+      <c r="F21" s="2">
         <v>20</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
+      <c r="G21" s="6">
+        <v>20</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B22" s="2">
         <v>1</v>
@@ -1018,13 +1088,16 @@
       <c r="E22" s="2">
         <v>1</v>
       </c>
-      <c r="F22" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
+      <c r="F22" s="2">
+        <v>1</v>
+      </c>
+      <c r="G22" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
       <c r="A23" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B23" s="2">
         <v>10</v>
@@ -1038,13 +1111,16 @@
       <c r="E23" s="2">
         <v>10</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="2">
         <v>10</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
+      <c r="G23" s="6">
+        <v>10</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
       <c r="A24" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B24" s="2">
         <v>200</v>
@@ -1058,13 +1134,16 @@
       <c r="E24" s="2">
         <v>200</v>
       </c>
-      <c r="F24" s="6">
+      <c r="F24" s="2">
         <v>200</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
+      <c r="G24" s="6">
+        <v>200</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
       <c r="A25" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B25" s="2">
         <v>1000</v>
@@ -1078,13 +1157,16 @@
       <c r="E25" s="2">
         <v>1000</v>
       </c>
-      <c r="F25" s="6">
+      <c r="F25" s="2">
         <v>1000</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
+      <c r="G25" s="6">
+        <v>1000</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
       <c r="A26" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B26" s="2">
         <v>1</v>
@@ -1098,13 +1180,16 @@
       <c r="E26" s="2">
         <v>1</v>
       </c>
-      <c r="F26" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
+      <c r="F26" s="2">
+        <v>1</v>
+      </c>
+      <c r="G26" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5">
       <c r="A27" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B27" s="2">
         <v>9</v>
@@ -1118,13 +1203,16 @@
       <c r="E27" s="2">
         <v>9</v>
       </c>
-      <c r="F27" s="6">
+      <c r="F27" s="2">
         <v>9</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
+      <c r="G27" s="6">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5">
       <c r="A28" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B28" s="9">
         <v>0.2</v>
@@ -1138,13 +1226,16 @@
       <c r="E28" s="9">
         <v>0.2</v>
       </c>
-      <c r="F28" s="10">
+      <c r="F28" s="9">
         <v>0.2</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
+      <c r="G28" s="10">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5">
       <c r="A29" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B29" s="9">
         <v>0.01</v>
@@ -1158,13 +1249,16 @@
       <c r="E29" s="9">
         <v>0.01</v>
       </c>
-      <c r="F29" s="10">
+      <c r="F29" s="9">
         <v>0.01</v>
       </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
+      <c r="G29" s="10">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5">
       <c r="A30" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B30" s="2">
         <v>1</v>
@@ -1178,13 +1272,16 @@
       <c r="E30" s="2">
         <v>1</v>
       </c>
-      <c r="F30" s="6">
+      <c r="F30" s="2">
+        <v>1</v>
+      </c>
+      <c r="G30" s="6">
         <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5">
       <c r="A31" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B31" s="9">
         <v>0.95</v>
@@ -1198,13 +1295,16 @@
       <c r="E31" s="9">
         <v>0.95</v>
       </c>
-      <c r="F31" s="10">
+      <c r="F31" s="9">
+        <v>0.95</v>
+      </c>
+      <c r="G31" s="10">
         <v>0.95</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="19.5">
       <c r="A32" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B32" s="2">
         <v>5</v>
@@ -1218,69 +1318,75 @@
       <c r="E32" s="2">
         <v>5</v>
       </c>
-      <c r="F32" s="6">
+      <c r="F32" s="2">
+        <v>5</v>
+      </c>
+      <c r="G32" s="6">
         <v>5</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="19.5">
       <c r="A33" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>43</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G33" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="19.5">
       <c r="A34" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C34" s="3" t="s">
-        <v>43</v>
-      </c>
       <c r="D34" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="F34" s="5" t="s">
-        <v>43</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G34" s="5"/>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="19.5">
       <c r="A35" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="F35" s="5" t="s">
         <v>51</v>
       </c>
+      <c r="E35" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G35" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>